<commit_message>
fix: proper "..." forwarding in SPatial_Extract feat: Spatial_Aggregate function feat: Spatial_Disaggregate function feat: NORA3 example data added fix: also document arguments of Viz_SpatRast in excel sheet now
</commit_message>
<xml_diff>
--- a/.github/ArgumentUsage.xlsx
+++ b/.github/ArgumentUsage.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cicero-my.sharepoint.com/personal/erikkus_cicero_oslo_no/Documents/Documents/31569 - ClimHub/ClimHub_GitHub/.github/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="86" documentId="8_{1892F552-129D-4505-A1EB-B37419729DC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{15F55AAC-3F36-4DC4-8BB1-A5CBCBE1C000}"/>
+  <xr:revisionPtr revIDLastSave="151" documentId="8_{1892F552-129D-4505-A1EB-B37419729DC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AE89A7F1-516C-49B2-94FA-85216BB0CF04}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{7ED2EDC4-BD5E-49E4-AE72-BC07D1D41013}"/>
+    <workbookView xWindow="28680" yWindow="-10275" windowWidth="38640" windowHeight="21120" xr2:uid="{7ED2EDC4-BD5E-49E4-AE72-BC07D1D41013}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="184">
   <si>
     <t>Argument</t>
   </si>
@@ -495,6 +495,99 @@
   </si>
   <si>
     <t>Access_reanalysis_cerra_single_levels</t>
+  </si>
+  <si>
+    <t>Viz_SpatRast</t>
+  </si>
+  <si>
+    <t>colour</t>
+  </si>
+  <si>
+    <t>legendTitle</t>
+  </si>
+  <si>
+    <t>panelLabels</t>
+  </si>
+  <si>
+    <t>panelColumns</t>
+  </si>
+  <si>
+    <t>sfObj</t>
+  </si>
+  <si>
+    <t>sfSize</t>
+  </si>
+  <si>
+    <t>sfShape</t>
+  </si>
+  <si>
+    <t>sfColour</t>
+  </si>
+  <si>
+    <t>sfFill</t>
+  </si>
+  <si>
+    <t>colour palette for raster plotting</t>
+  </si>
+  <si>
+    <t>title for colour legend in plot</t>
+  </si>
+  <si>
+    <t>title for panels in plot</t>
+  </si>
+  <si>
+    <t>how many columns to arrange plot panels in</t>
+  </si>
+  <si>
+    <t>sf object to overlay in plot</t>
+  </si>
+  <si>
+    <t>size of plotting of sf object</t>
+  </si>
+  <si>
+    <t>shape of plotting of sf object</t>
+  </si>
+  <si>
+    <t>colour of plotting of sf object</t>
+  </si>
+  <si>
+    <t>fill colour of plotting of sf object</t>
+  </si>
+  <si>
+    <t>…</t>
+  </si>
+  <si>
+    <t>additional arguments passed further down</t>
+  </si>
+  <si>
+    <t>Spatial_Aggregate</t>
+  </si>
+  <si>
+    <t>factor</t>
+  </si>
+  <si>
+    <t>spatRasterFrom</t>
+  </si>
+  <si>
+    <t>spatRasterTo</t>
+  </si>
+  <si>
+    <t>numeric factor for (dis-)aggregation</t>
+  </si>
+  <si>
+    <t>spatRaster from which to do an operation</t>
+  </si>
+  <si>
+    <t>spatRaster to which an operation from another ought to match</t>
+  </si>
+  <si>
+    <t>Spatial_Disaggregate</t>
+  </si>
+  <si>
+    <t>Helper_PolySummary</t>
+  </si>
+  <si>
+    <t>Helper_AttrOverride</t>
   </si>
 </sst>
 </file>
@@ -544,12 +637,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -885,107 +977,122 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{07D92B5E-1B5B-4594-8844-F2047C5EAE1B}">
-  <dimension ref="A1:AD62"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:AI75"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="19.140625" style="2" customWidth="1"/>
-    <col min="2" max="5" width="44.42578125" customWidth="1"/>
-    <col min="6" max="6" width="18.42578125" customWidth="1"/>
+    <col min="1" max="1" width="19.109375" customWidth="1"/>
+    <col min="2" max="2" width="44.44140625" customWidth="1"/>
+    <col min="3" max="35" width="2.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:35" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="2" t="s">
         <v>151</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="H1" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="I1" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="J1" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="K1" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="L1" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="M1" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="N1" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="O1" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="P1" s="3" t="s">
+      <c r="P1" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="Q1" s="3" t="s">
+      <c r="Q1" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="R1" s="3" t="s">
+      <c r="R1" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="S1" s="3" t="s">
+      <c r="S1" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="T1" s="3" t="s">
+      <c r="T1" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="U1" s="3" t="s">
+      <c r="U1" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="V1" s="3" t="s">
+      <c r="V1" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="W1" s="3" t="s">
+      <c r="W1" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="X1" s="3" t="s">
+      <c r="X1" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="Y1" s="3" t="s">
+      <c r="Y1" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="Z1" s="3" t="s">
+      <c r="Z1" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="AA1" s="3" t="s">
+      <c r="AA1" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="AB1" s="3" t="s">
+      <c r="AB1" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="AC1" s="3" t="s">
+      <c r="AC1" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="AD1" s="3" t="s">
+      <c r="AD1" s="2" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="AE1" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="AF1" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="AG1" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="AH1" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="AI1" s="2" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="2" spans="1:35" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -1013,8 +1120,11 @@
       <c r="AC2" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="3" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="AE2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:35" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
@@ -1046,7 +1156,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
@@ -1057,7 +1167,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>7</v>
       </c>
@@ -1068,7 +1178,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>10</v>
       </c>
@@ -1079,7 +1189,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>12</v>
       </c>
@@ -1090,7 +1200,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:35" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>11</v>
       </c>
@@ -1101,7 +1211,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="9" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:35" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>18</v>
       </c>
@@ -1136,7 +1246,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:35" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>22</v>
       </c>
@@ -1147,7 +1257,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="11" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>24</v>
       </c>
@@ -1158,7 +1268,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="12" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>28</v>
       </c>
@@ -1169,7 +1279,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="13" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>29</v>
       </c>
@@ -1180,7 +1290,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="14" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>30</v>
       </c>
@@ -1202,8 +1312,11 @@
       <c r="O14" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="15" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="AF14" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="15" spans="1:35" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>35</v>
       </c>
@@ -1217,7 +1330,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="16" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:35" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>36</v>
       </c>
@@ -1228,7 +1341,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="17" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:34" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>37</v>
       </c>
@@ -1244,8 +1357,17 @@
       <c r="P17" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="18" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="AF17" t="s">
+        <v>17</v>
+      </c>
+      <c r="AG17" t="s">
+        <v>17</v>
+      </c>
+      <c r="AH17" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="18" spans="1:34" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
         <v>41</v>
       </c>
@@ -1256,7 +1378,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:34" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
         <v>42</v>
       </c>
@@ -1267,7 +1389,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="20" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:34" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
         <v>47</v>
       </c>
@@ -1278,7 +1400,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="21" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:34" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
         <v>48</v>
       </c>
@@ -1289,7 +1411,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="22" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:34" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
         <v>49</v>
       </c>
@@ -1300,7 +1422,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="23" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:34" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
         <v>50</v>
       </c>
@@ -1311,7 +1433,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="24" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:34" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
         <v>56</v>
       </c>
@@ -1325,7 +1447,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="25" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:34" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
         <v>59</v>
       </c>
@@ -1336,7 +1458,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="26" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:34" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
         <v>62</v>
       </c>
@@ -1347,7 +1469,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="27" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:34" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
         <v>63</v>
       </c>
@@ -1358,7 +1480,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="28" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:34" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
         <v>64</v>
       </c>
@@ -1369,7 +1491,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="29" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:34" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
         <v>70</v>
       </c>
@@ -1383,7 +1505,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="30" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:34" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
         <v>73</v>
       </c>
@@ -1394,7 +1516,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="31" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:34" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
         <v>76</v>
       </c>
@@ -1405,7 +1527,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="32" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:34" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
         <v>79</v>
       </c>
@@ -1416,7 +1538,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="33" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
         <v>80</v>
       </c>
@@ -1427,7 +1549,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="34" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
         <v>83</v>
       </c>
@@ -1441,7 +1563,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="35" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
         <v>84</v>
       </c>
@@ -1455,7 +1577,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="36" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
         <v>85</v>
       </c>
@@ -1466,7 +1588,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="37" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
         <v>86</v>
       </c>
@@ -1477,7 +1599,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="38" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
         <v>87</v>
       </c>
@@ -1488,7 +1610,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="39" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A39" s="1" t="s">
         <v>88</v>
       </c>
@@ -1499,7 +1621,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="40" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
         <v>89</v>
       </c>
@@ -1510,7 +1632,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="41" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
         <v>58</v>
       </c>
@@ -1521,7 +1643,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="42" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A42" s="1" t="s">
         <v>90</v>
       </c>
@@ -1532,7 +1654,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="43" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A43" s="1" t="s">
         <v>96</v>
       </c>
@@ -1543,7 +1665,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="44" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
         <v>108</v>
       </c>
@@ -1557,7 +1679,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="45" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A45" s="1" t="s">
         <v>112</v>
       </c>
@@ -1568,7 +1690,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="46" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A46" s="1" t="s">
         <v>113</v>
       </c>
@@ -1579,7 +1701,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="47" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A47" s="1" t="s">
         <v>114</v>
       </c>
@@ -1590,7 +1712,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="48" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A48" s="1" t="s">
         <v>121</v>
       </c>
@@ -1601,7 +1723,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A49" s="1" t="s">
         <v>123</v>
       </c>
@@ -1618,7 +1740,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A50" s="1" t="s">
         <v>124</v>
       </c>
@@ -1635,7 +1757,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A51" s="1" t="s">
         <v>125</v>
       </c>
@@ -1652,7 +1774,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A52" s="1" t="s">
         <v>126</v>
       </c>
@@ -1663,7 +1785,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A53" s="1" t="s">
         <v>127</v>
       </c>
@@ -1674,7 +1796,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A54" s="1" t="s">
         <v>128</v>
       </c>
@@ -1691,7 +1813,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A55" s="1" t="s">
         <v>129</v>
       </c>
@@ -1708,7 +1830,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A56" s="1" t="s">
         <v>130</v>
       </c>
@@ -1719,7 +1841,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A57" s="1" t="s">
         <v>131</v>
       </c>
@@ -1730,7 +1852,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A58" s="1" t="s">
         <v>132</v>
       </c>
@@ -1741,7 +1863,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A59" s="1" t="s">
         <v>133</v>
       </c>
@@ -1752,7 +1874,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A60" s="1" t="s">
         <v>134</v>
       </c>
@@ -1763,7 +1885,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A61" s="1" t="s">
         <v>135</v>
       </c>
@@ -1777,7 +1899,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A62" s="1" t="s">
         <v>136</v>
       </c>
@@ -1785,6 +1907,179 @@
         <v>144</v>
       </c>
       <c r="E62" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="63" spans="1:31" x14ac:dyDescent="0.3">
+      <c r="A63" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="B63" t="s">
+        <v>163</v>
+      </c>
+      <c r="AE63" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="64" spans="1:31" x14ac:dyDescent="0.3">
+      <c r="A64" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="B64" t="s">
+        <v>164</v>
+      </c>
+      <c r="AE64" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="65" spans="1:35" x14ac:dyDescent="0.3">
+      <c r="A65" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="B65" t="s">
+        <v>165</v>
+      </c>
+      <c r="AE65" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="66" spans="1:35" x14ac:dyDescent="0.3">
+      <c r="A66" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="B66" t="s">
+        <v>166</v>
+      </c>
+      <c r="AE66" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="67" spans="1:35" x14ac:dyDescent="0.3">
+      <c r="A67" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="B67" t="s">
+        <v>167</v>
+      </c>
+      <c r="AE67" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="68" spans="1:35" x14ac:dyDescent="0.3">
+      <c r="A68" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="B68" t="s">
+        <v>168</v>
+      </c>
+      <c r="AE68" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="69" spans="1:35" x14ac:dyDescent="0.3">
+      <c r="A69" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="B69" t="s">
+        <v>169</v>
+      </c>
+      <c r="AE69" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="70" spans="1:35" x14ac:dyDescent="0.3">
+      <c r="A70" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="B70" t="s">
+        <v>170</v>
+      </c>
+      <c r="AE70" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="71" spans="1:35" x14ac:dyDescent="0.3">
+      <c r="A71" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="B71" t="s">
+        <v>171</v>
+      </c>
+      <c r="AE71" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="72" spans="1:35" x14ac:dyDescent="0.3">
+      <c r="A72" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="B72" t="s">
+        <v>173</v>
+      </c>
+      <c r="P72" t="s">
+        <v>17</v>
+      </c>
+      <c r="AF72" t="s">
+        <v>17</v>
+      </c>
+      <c r="AG72" t="s">
+        <v>17</v>
+      </c>
+      <c r="AH72" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="73" spans="1:35" x14ac:dyDescent="0.3">
+      <c r="A73" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="B73" t="s">
+        <v>178</v>
+      </c>
+      <c r="AF73" t="s">
+        <v>17</v>
+      </c>
+      <c r="AG73" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="74" spans="1:35" x14ac:dyDescent="0.3">
+      <c r="A74" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="B74" t="s">
+        <v>179</v>
+      </c>
+      <c r="AF74" t="s">
+        <v>17</v>
+      </c>
+      <c r="AG74" t="s">
+        <v>17</v>
+      </c>
+      <c r="AH74" t="s">
+        <v>17</v>
+      </c>
+      <c r="AI74" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="75" spans="1:35" x14ac:dyDescent="0.3">
+      <c r="A75" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="B75" t="s">
+        <v>180</v>
+      </c>
+      <c r="AF75" t="s">
+        <v>17</v>
+      </c>
+      <c r="AG75" t="s">
+        <v>17</v>
+      </c>
+      <c r="AH75" t="s">
+        <v>17</v>
+      </c>
+      <c r="AI75" t="s">
         <v>17</v>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: refresh ArgumentUsage workbook
</commit_message>
<xml_diff>
--- a/.github/ArgumentUsage.xlsx
+++ b/.github/ArgumentUsage.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="368" uniqueCount="215">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="242">
   <si>
     <t>Argument</t>
   </si>
@@ -169,6 +169,15 @@
     <t>Helper_VarDFtoJSON</t>
   </si>
   <si>
+    <t>Helper_ETCCDIDailyBootstraps</t>
+  </si>
+  <si>
+    <t>Helper_ETCCDIGSL</t>
+  </si>
+  <si>
+    <t>Metrics_BootstrapQuantiles</t>
+  </si>
+  <si>
     <t>spatRaster</t>
   </si>
   <si>
@@ -680,6 +689,78 @@
   </si>
   <si>
     <t>Character string with the path to the output JSON file.</t>
+  </si>
+  <si>
+    <t>CFVariable</t>
+  </si>
+  <si>
+    <t>A CFVariable object to be processed.</t>
+  </si>
+  <si>
+    <t>threshMode</t>
+  </si>
+  <si>
+    <t>Character, optional. If supplying a CFVariable containing baseline quantiles for ETCCDI calculation, setting threshMode = "ETCCDIQuantiles" will internally apply location and day-of-year specific thresholds to CFVariable input. Default is NULL avoiding this behaviour.</t>
+  </si>
+  <si>
+    <t>returnSummary</t>
+  </si>
+  <si>
+    <t>Function. Summary function for tresholded CFVariable.</t>
+  </si>
+  <si>
+    <t>returnTResolution</t>
+  </si>
+  <si>
+    <t>Character. Temporal resolution of summary of tresholded CFVariable.</t>
+  </si>
+  <si>
+    <t>projectionList</t>
+  </si>
+  <si>
+    <t>List. List of CFVariable objects required by the selected ETCCDI indices via the indices argument. Include only named elements that are needed for indices: "TX" (daily maximum air temperature in Kelvin), "TN" (daily minimum air temperature in Kelvin), and/or "RR" (daily total precipitation in mm). See details for required data input per index.</t>
+  </si>
+  <si>
+    <t>baseLineList</t>
+  </si>
+  <si>
+    <t>Optional, list. List of CFDataset objects containing baseline quantiles required only for quantile-based ETCCDI indices. Include only named elements needed for indices: "TX_Base", "TN_Base", and/or "RR_Base" (note that these must be in Kelvin, Kelvin, and mm, respectively). If no quantile-based ETCCDI is selected, this argument can be omitted. See details for required quantile baselines per index.</t>
+  </si>
+  <si>
+    <t>indices</t>
+  </si>
+  <si>
+    <t>Optional, character. Character vector of ETCCDI abbreviations to calculate (see first column of the details table). If missing, all supported indices in this function are calculated. See details for supported indices.</t>
+  </si>
+  <si>
+    <t>TResolution</t>
+  </si>
+  <si>
+    <t>Optional, character. Temporal resolution for ETCCDI calculation. Supports "year", "month" and "season". If omitted, each selected index is calculated using its default temporal resolution from the details table. If provided, the same resolution is used for all selected indices and output indices whose default resolution differs are prefixed with "ALT_". Note that this is not applied to GSL which is always calculated at annual resolution due to its specific logic.</t>
+  </si>
+  <si>
+    <t>RRThreshold</t>
+  </si>
+  <si>
+    <t>Numeric. Custom threshold for daily precipiation in mm for calculation of Rnnmm. Defaults to 42.</t>
+  </si>
+  <si>
+    <t>bootstrapWindow</t>
+  </si>
+  <si>
+    <t>Numeric/Integer. Shared argument reused across package functions; see function-specific help for exact behaviour.</t>
+  </si>
+  <si>
+    <t>TM</t>
+  </si>
+  <si>
+    <t>A CFVariable containing daily mean temperatures (or similar) to be used for GSL calculation.</t>
+  </si>
+  <si>
+    <t>probs</t>
+  </si>
+  <si>
+    <t>Numeric vector of probabilities (between 0 and 1) for which quantiles will be returned. Default is c(0.1,0.9).</t>
   </si>
 </sst>
 </file>
@@ -1069,15 +1150,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{07D92B5E-1B5B-4594-8844-F2047C5EAE1B}">
-  <dimension ref="A1:AR86"/>
+  <dimension ref="A1:AU98"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="19.109375" customWidth="1"/>
     <col min="2" max="2" width="44.44140625" customWidth="1"/>
-    <col min="3" max="44" width="2.77734375" customWidth="1"/>
+    <col min="3" max="47" width="2.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:44" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:47" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1210,1147 +1291,1291 @@
       <c r="AR1" s="2" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="2" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="AS1" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="AT1" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="AU1" s="2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="2" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="B2" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="F2" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="I2" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="J2" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="P2" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="R2" t="s">
-        <v>46</v>
-      </c>
-      <c r="AA2" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="AC2" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="AK2" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="3" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="3" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="B3" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="C3" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="D3" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="E3" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="F3" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="G3" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="H3" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="O3" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="Y3" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="4" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+      <c r="AB3" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="4" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="B4" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="F4" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="5" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="5" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="B5" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="F5" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="6" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="6" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="B6" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="F6" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="7" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="7" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="B7" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="F7" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="8" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="8" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B8" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C8" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="D8" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="E8" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="F8" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="9" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="9" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="B9" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="F9" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="H9" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="I9" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="J9" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="L9" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="M9" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="O9" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="R9" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="Y9" t="s">
-        <v>46</v>
-      </c>
-      <c r="AA9" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="AP9" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="10" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="10" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="B10" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="H10" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="11" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="11" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="B11" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="H11" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="12" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="12" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="B12" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="I12" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="13" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="13" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="B13" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="I13" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="14" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="14" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="B14" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="I14" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="L14" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="O14" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="AL14" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="15" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="15" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="B15" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="J15" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="AC15" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="16" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="16" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="B16" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="J16" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="17" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="17" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="B17" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="J17" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="M17" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="P17" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="AL17" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="AM17" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="AN17" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="18" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="18" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="B18" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="K18" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="19" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="19" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="B19" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="K19" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="20" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="20" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="B20" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="L20" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="21" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="21" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="B21" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="L21" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="22" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="22" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B22" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="L22" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="23" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="23" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="B23" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="L23" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="24" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="24" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="B24" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="M24" t="s">
-        <v>46</v>
-      </c>
-      <c r="AB24" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="25" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="25" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="B25" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="O25" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="26" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="26" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="B26" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="N26" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="27" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="27" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="B27" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="N27" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="28" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="28" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="B28" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="N28" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="29" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="29" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="B29" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="P29" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="Q29" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="30" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="30" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="B30" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="Q30" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="31" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="31" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="B31" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="R31" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="32" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="32" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="B32" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="S32" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="33" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="33" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="B33" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="S33" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="34" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="34" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="B34" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="E34" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="T34" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="W34" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="35" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="35" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="B35" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="E35" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="T35" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="W35" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="36" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="36" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="B36" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="U36" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="37" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="37" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="B37" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="U37" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="38" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="38" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="B38" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="E38" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="U38" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="39" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="39" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A39" s="1" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B39" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="V39" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="40" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="40" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="B40" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="V40" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="41" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="41" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="B41" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="V41" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="42" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="42" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A42" s="1" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="B42" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="W42" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="43" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="43" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A43" s="1" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="B43" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="X43" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="44" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="44" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="B44" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="Y44" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="Z44" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="45" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+      <c r="AS44" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="45" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A45" s="1" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="B45" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="AA45" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="46" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="46" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A46" s="1" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="B46" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="AA46" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="47" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="47" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A47" s="1" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="B47" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="AA47" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="48" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="48" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A48" s="1" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="B48" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="AD48" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="AE48" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="AF48" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="AG48" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="AI48" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="AJ48" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="49" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="49" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A49" s="1" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="B49" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="C49" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="D49" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="E49" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="AP49" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="50" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="50" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A50" s="1" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="B50" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="C50" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="D50" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="E50" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="51" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="51" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A51" s="1" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="B51" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="C51" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="D51" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="E51" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="52" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="52" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A52" s="1" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="B52" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="C52" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="53" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="53" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A53" s="1" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="B53" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="C53" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="54" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="54" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A54" s="1" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="B54" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="E54" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="55" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="55" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A55" s="1" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="B55" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="E55" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="56" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="56" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A56" s="1" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="B56" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="E56" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="57" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="57" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A57" s="1" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="B57" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="E57" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="58" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="58" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A58" s="1" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="B58" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="E58" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="59" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="59" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A59" s="1" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="B59" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="E59" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="60" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="60" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A60" s="1" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="B60" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="E60" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="61" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="61" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A61" s="1" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="B61" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="D61" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="E61" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="62" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="62" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A62" s="1" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="B62" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="E62" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="63" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="63" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A63" s="1" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="B63" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="AK63" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="64" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="64" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A64" s="1" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="B64" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="AK64" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="65" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="65" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A65" s="1" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="B65" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="AK65" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="66" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="66" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A66" s="1" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="B66" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="AK66" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="67" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="67" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A67" s="1" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="B67" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="AK67" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="68" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="68" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A68" s="1" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="B68" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="AK68" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="69" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="69" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A69" s="1" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="B69" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="AK69" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="70" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="70" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A70" s="1" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="B70" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="AK70" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="71" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="71" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A71" s="1" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="B71" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="AK71" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="72" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="72" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A72" s="1" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="B72" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="G72" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="P72" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="AL72" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="AM72" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="AN72" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="73" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="73" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A73" s="1" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="B73" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="AL73" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="AM73" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="74" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="74" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A74" s="1" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="B74" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="AL74" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="AM74" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="AN74" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="AO74" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="75" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="75" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A75" s="1" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="B75" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="AL75" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="AM75" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="AN75" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="AO75" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="76" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="76" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A76" s="1" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="B76" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="C76" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="D76" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="77" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="77" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A77" s="1" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="B77" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="C77" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="78" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="78" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A78" s="1" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="B78" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="G78" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="79" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="79" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A79" s="1" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="B79" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="G79" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="80" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="80" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A80" s="1" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="B80" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="AP80" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="81" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="81" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A81" s="1" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="B81" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="AP81" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="82" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="82" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A82" s="1" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="B82" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="AQ82" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="83" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="83" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A83" s="1" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="B83" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="AQ83" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="84" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="84" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A84" s="1" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="B84" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="AQ84" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="85" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="85" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A85" s="1" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="B85" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="AR85" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="86" spans="1:44" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="86" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A86" s="1" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="B86" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="AR86" t="s">
-        <v>46</v>
+        <v>49</v>
+      </c>
+    </row>
+    <row r="87" spans="1:47" x14ac:dyDescent="0.3">
+      <c r="A87" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="B87" t="s">
+        <v>219</v>
+      </c>
+      <c r="AA87" t="s">
+        <v>49</v>
+      </c>
+      <c r="AU87" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="88" spans="1:47" x14ac:dyDescent="0.3">
+      <c r="A88" s="1" t="s">
+        <v>220</v>
+      </c>
+      <c r="B88" t="s">
+        <v>221</v>
+      </c>
+      <c r="AA88" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="89" spans="1:47" x14ac:dyDescent="0.3">
+      <c r="A89" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="B89" t="s">
+        <v>223</v>
+      </c>
+      <c r="AA89" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="90" spans="1:47" x14ac:dyDescent="0.3">
+      <c r="A90" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="B90" t="s">
+        <v>225</v>
+      </c>
+      <c r="AA90" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="91" spans="1:47" x14ac:dyDescent="0.3">
+      <c r="A91" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="B91" t="s">
+        <v>227</v>
+      </c>
+      <c r="AB91" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="92" spans="1:47" x14ac:dyDescent="0.3">
+      <c r="A92" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="B92" t="s">
+        <v>229</v>
+      </c>
+      <c r="AB92" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="93" spans="1:47" x14ac:dyDescent="0.3">
+      <c r="A93" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="B93" t="s">
+        <v>231</v>
+      </c>
+      <c r="AB93" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="94" spans="1:47" x14ac:dyDescent="0.3">
+      <c r="A94" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="B94" t="s">
+        <v>233</v>
+      </c>
+      <c r="AB94" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="95" spans="1:47" x14ac:dyDescent="0.3">
+      <c r="A95" s="1" t="s">
+        <v>234</v>
+      </c>
+      <c r="B95" t="s">
+        <v>235</v>
+      </c>
+      <c r="AB95" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="96" spans="1:47" x14ac:dyDescent="0.3">
+      <c r="A96" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="B96" t="s">
+        <v>237</v>
+      </c>
+      <c r="AS96" t="s">
+        <v>49</v>
+      </c>
+      <c r="AU96" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="97" spans="1:47" x14ac:dyDescent="0.3">
+      <c r="A97" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="B97" t="s">
+        <v>239</v>
+      </c>
+      <c r="AT97" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="98" spans="1:47" x14ac:dyDescent="0.3">
+      <c r="A98" s="1" t="s">
+        <v>240</v>
+      </c>
+      <c r="B98" t="s">
+        <v>241</v>
+      </c>
+      <c r="AU98" t="s">
+        <v>49</v>
       </c>
     </row>
   </sheetData>

</xml_diff>